<commit_message>
Record glassine bag standard cost £0.09686 in trims list
Consolidate the two glassine bag lines into one item, fill in its Sage
code PKG-BAG-GLA-68x92-PS and unit cost 0.09686 across the trims master
workbook and CSVs; confirmed codes/costs now persist through regeneration.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016cXYvn1BQCe2wgwE2RjU2a
</commit_message>
<xml_diff>
--- a/trims-master.xlsx
+++ b/trims-master.xlsx
@@ -13,7 +13,7 @@
     <sheet name="By style" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sage codes to create'!$A$1:$F$174</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sage codes to create'!$A$1:$F$173</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trims master'!$A$1:$H$573</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'By style'!$A$1:$H$1462</definedName>
   </definedNames>
@@ -23,7 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="£0.00000"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -98,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -109,6 +111,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -512,7 +517,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Those lines mostly differ only by placement wording, so they are also consolidated into 173 suggested purchasable items.</t>
+          <t>Those lines mostly differ only by placement wording, so they are also consolidated into 172 suggested purchasable items.</t>
         </is>
       </c>
     </row>
@@ -616,7 +621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F174"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4042,7 +4047,7 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
@@ -4051,23 +4056,29 @@
         </is>
       </c>
       <c r="C171" s="4" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D171" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E171" s="5" t="inlineStr"/>
-      <c r="F171" s="5" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>PKG-BAG-GLA-68x92-PS</t>
+        </is>
+      </c>
+      <c r="F171" s="6" t="n">
+        <v>0.09686</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Antique brass 15mm cap (parts a and b)</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="C172" s="4" t="n">
@@ -4082,7 +4093,7 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>Antique brass 15mm cap (parts a and b)</t>
+          <t>Oliver harvey</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
@@ -4091,7 +4102,7 @@
         </is>
       </c>
       <c r="C173" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D173" s="4" t="n">
         <v>1</v>
@@ -4099,28 +4110,8 @@
       <c r="E173" s="5" t="inlineStr"/>
       <c r="F173" s="5" t="inlineStr"/>
     </row>
-    <row r="174">
-      <c r="A174" s="4" t="inlineStr">
-        <is>
-          <t>Oliver harvey</t>
-        </is>
-      </c>
-      <c r="B174" s="4" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C174" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D174" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E174" s="5" t="inlineStr"/>
-      <c r="F174" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F174"/>
+  <autoFilter ref="A1:F173"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18837,7 +18828,7 @@
           <t>Tax tabs</t>
         </is>
       </c>
-      <c r="C368" s="6" t="inlineStr">
+      <c r="C368" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -18873,7 +18864,7 @@
           <t>Tax tabs</t>
         </is>
       </c>
-      <c r="C369" s="6" t="inlineStr">
+      <c r="C369" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -25745,7 +25736,7 @@
           <t>Care / wash labels</t>
         </is>
       </c>
-      <c r="C541" s="6" t="inlineStr">
+      <c r="C541" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -25781,7 +25772,7 @@
           <t>Care / wash labels</t>
         </is>
       </c>
-      <c r="C542" s="6" t="inlineStr">
+      <c r="C542" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -25817,7 +25808,7 @@
           <t>Care / wash labels</t>
         </is>
       </c>
-      <c r="C543" s="6" t="inlineStr">
+      <c r="C543" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26420,25 +26411,25 @@
       </c>
       <c r="D558" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E558" s="4" t="inlineStr">
         <is>
-          <t>Glassine Bag for packing</t>
+          <t>Glassine bag for packing — PKG-BAG-GLA-68x92-PS</t>
         </is>
       </c>
       <c r="F558" s="4" t="inlineStr">
         <is>
-          <t>GLASSINE PEEL &amp; SEAL BIODEGRADABLE BAG (68x92cm) ref - PKG-BAG-GLA-68x92-PS Supplier Glassine Bags - on line</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="G558" s="4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="H558" s="4" t="inlineStr">
         <is>
-          <t>OHTAB222/LT</t>
+          <t>OHTAB921; OHTAB01; OHTAB03; OHTAB04; OHTAB06; OHTAB11; OHTAB14; OHTAB15; OHTAB24; OHTAB82; OHTAB83; OHTAB131; OHTAB286</t>
         </is>
       </c>
     </row>
@@ -26460,25 +26451,25 @@
       </c>
       <c r="D559" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E559" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — PKG-BAG-GLA-68x92-PS</t>
+          <t>Glassine Bag for packing</t>
         </is>
       </c>
       <c r="F559" s="4" t="inlineStr">
         <is>
-          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
+          <t>GLASSINE PEEL &amp; SEAL BIODEGRADABLE BAG (68x92cm) ref - PKG-BAG-GLA-68x92-PS Supplier Glassine Bags - on line</t>
         </is>
       </c>
       <c r="G559" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="H559" s="4" t="inlineStr">
         <is>
-          <t>OHTAB921; OHTAB01; OHTAB03; OHTAB04; OHTAB06; OHTAB11; OHTAB14; OHTAB15; OHTAB24; OHTAB82; OHTAB83; OHTAB131; OHTAB286</t>
+          <t>OHTAB222/LT</t>
         </is>
       </c>
     </row>
@@ -26573,7 +26564,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C562" s="6" t="inlineStr">
+      <c r="C562" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26609,7 +26600,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C563" s="6" t="inlineStr">
+      <c r="C563" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26645,7 +26636,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C564" s="6" t="inlineStr">
+      <c r="C564" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26681,7 +26672,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C565" s="6" t="inlineStr">
+      <c r="C565" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26717,7 +26708,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C566" s="6" t="inlineStr">
+      <c r="C566" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26753,7 +26744,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C567" s="6" t="inlineStr">
+      <c r="C567" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26789,7 +26780,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C568" s="6" t="inlineStr">
+      <c r="C568" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26825,7 +26816,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C569" s="6" t="inlineStr">
+      <c r="C569" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26861,7 +26852,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C570" s="6" t="inlineStr">
+      <c r="C570" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26897,7 +26888,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C571" s="6" t="inlineStr">
+      <c r="C571" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26933,7 +26924,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C572" s="6" t="inlineStr">
+      <c r="C572" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -26969,7 +26960,7 @@
           <t>Spec / info only</t>
         </is>
       </c>
-      <c r="C573" s="6" t="inlineStr">
+      <c r="C573" s="7" t="inlineStr">
         <is>
           <t>Spec note</t>
         </is>
@@ -55002,12 +54993,12 @@
       </c>
       <c r="C822" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D822" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E822" s="4" t="inlineStr">
@@ -55176,12 +55167,12 @@
       </c>
       <c r="C827" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D827" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E827" s="4" t="inlineStr">
@@ -55350,12 +55341,12 @@
       </c>
       <c r="C832" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D832" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E832" s="4" t="inlineStr">
@@ -55524,12 +55515,12 @@
       </c>
       <c r="C837" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D837" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E837" s="4" t="inlineStr">
@@ -55698,12 +55689,12 @@
       </c>
       <c r="C842" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D842" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E842" s="4" t="inlineStr">
@@ -55872,12 +55863,12 @@
       </c>
       <c r="C847" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D847" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E847" s="4" t="inlineStr">
@@ -56046,12 +56037,12 @@
       </c>
       <c r="C852" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D852" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E852" s="4" t="inlineStr">
@@ -56220,12 +56211,12 @@
       </c>
       <c r="C857" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D857" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E857" s="4" t="inlineStr">
@@ -56394,12 +56385,12 @@
       </c>
       <c r="C862" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D862" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E862" s="4" t="inlineStr">
@@ -56568,12 +56559,12 @@
       </c>
       <c r="C867" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D867" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E867" s="4" t="inlineStr">
@@ -56742,12 +56733,12 @@
       </c>
       <c r="C872" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D872" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E872" s="4" t="inlineStr">
@@ -56916,12 +56907,12 @@
       </c>
       <c r="C877" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D877" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E877" s="4" t="inlineStr">
@@ -57090,12 +57081,12 @@
       </c>
       <c r="C882" s="4" t="inlineStr">
         <is>
-          <t>T558</t>
+          <t>T557</t>
         </is>
       </c>
       <c r="D882" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing — pkg-bag-gla-68</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E882" s="4" t="inlineStr">
@@ -57124,12 +57115,12 @@
       </c>
       <c r="C883" s="4" t="inlineStr">
         <is>
-          <t>T557</t>
+          <t>T558</t>
         </is>
       </c>
       <c r="D883" s="4" t="inlineStr">
         <is>
-          <t>Glassine bag for packing</t>
+          <t>Glassine peel &amp; seal biodegradable bag (68x92cm)</t>
         </is>
       </c>
       <c r="E883" s="4" t="inlineStr">

</xml_diff>